<commit_message>
Actualización: agregué nuevas funciones
</commit_message>
<xml_diff>
--- a/Documentacion/HISTORIAS DE USUARIOS PanApp.xlsx
+++ b/Documentacion/HISTORIAS DE USUARIOS PanApp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexander Otalora\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\PanApp\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D54638-CD48-4452-BE9E-FFE7C1F25F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B55FCF6-C8E7-4BB9-BA7B-4727733F073D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1078,23 +1078,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1103,34 +1122,15 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1364,18 +1364,18 @@
   <sheetData>
     <row r="1" spans="1:9" ht="14.25" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="41" t="s">
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="42"/>
     </row>
     <row r="2" spans="1:9" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1407,16 +1407,16 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="38" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="3">
@@ -1436,10 +1436,10 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
       <c r="E4" s="3">
         <v>2</v>
       </c>
@@ -1457,42 +1457,42 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="37.5" customHeight="1">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="33">
+      <c r="A5" s="43"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44">
         <v>3</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="35" t="s">
+      <c r="G5" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="35" t="s">
+      <c r="H5" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="35" t="s">
+      <c r="I5" s="38" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A6" s="31"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
     </row>
     <row r="7" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A7" s="32"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
       <c r="E7" s="6">
         <v>4</v>
       </c>
@@ -1521,16 +1521,16 @@
       <c r="I8" s="7"/>
     </row>
     <row r="9" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="38" t="s">
         <v>34</v>
       </c>
       <c r="E9" s="3">
@@ -1550,10 +1550,10 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="3">
         <v>2</v>
       </c>
@@ -1571,42 +1571,42 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A11" s="31"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="33">
+      <c r="A11" s="43"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44">
         <v>3</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="35" t="s">
+      <c r="G11" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="35" t="s">
+      <c r="H11" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="35" t="s">
+      <c r="I11" s="38" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
+      <c r="A12" s="43"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
     </row>
     <row r="13" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A13" s="32"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
       <c r="E13" s="8"/>
       <c r="F13" s="6"/>
       <c r="G13" s="4"/>
@@ -1625,16 +1625,16 @@
       <c r="I14" s="7"/>
     </row>
     <row r="15" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="38" t="s">
         <v>48</v>
       </c>
       <c r="E15" s="3">
@@ -1654,10 +1654,10 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A16" s="31"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
+      <c r="A16" s="43"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
       <c r="E16" s="3">
         <v>2</v>
       </c>
@@ -1675,42 +1675,42 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A17" s="31"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="33">
+      <c r="A17" s="43"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="44">
         <v>3</v>
       </c>
-      <c r="F17" s="35" t="s">
+      <c r="F17" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="35" t="s">
+      <c r="G17" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="H17" s="35" t="s">
+      <c r="H17" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="I17" s="35" t="s">
+      <c r="I17" s="38" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A18" s="31"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
+      <c r="A18" s="43"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
+      <c r="A19" s="39"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
       <c r="E19" s="6">
         <v>4</v>
       </c>
@@ -1739,16 +1739,16 @@
       <c r="I20" s="13"/>
     </row>
     <row r="21" spans="1:10" ht="43.2">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="D21" s="35" t="s">
+      <c r="D21" s="38" t="s">
         <v>67</v>
       </c>
       <c r="E21" s="12">
@@ -1768,10 +1768,10 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="45" customHeight="1">
-      <c r="A22" s="31"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
+      <c r="A22" s="43"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
       <c r="E22" s="12">
         <v>2</v>
       </c>
@@ -1790,43 +1790,43 @@
       <c r="J22" s="11"/>
     </row>
     <row r="23" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A23" s="31"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="33">
+      <c r="A23" s="43"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44">
         <v>3</v>
       </c>
-      <c r="F23" s="36" t="s">
+      <c r="F23" s="50" t="s">
         <v>203</v>
       </c>
-      <c r="G23" s="36" t="s">
+      <c r="G23" s="50" t="s">
         <v>204</v>
       </c>
-      <c r="H23" s="36" t="s">
+      <c r="H23" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="I23" s="36" t="s">
+      <c r="I23" s="50" t="s">
         <v>206</v>
       </c>
       <c r="J23" s="11"/>
     </row>
     <row r="24" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A24" s="31"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
+      <c r="A24" s="43"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
     </row>
     <row r="25" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A25" s="32"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
+      <c r="A25" s="39"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -1845,16 +1845,16 @@
       <c r="I26" s="7"/>
     </row>
     <row r="27" spans="1:10" ht="28.5" customHeight="1">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C27" s="35" t="s">
+      <c r="C27" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="38" t="s">
         <v>72</v>
       </c>
       <c r="E27" s="3">
@@ -1874,10 +1874,10 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A28" s="31"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
+      <c r="A28" s="43"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
       <c r="E28" s="3">
         <v>2</v>
       </c>
@@ -1895,42 +1895,42 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A29" s="31"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="33">
+      <c r="A29" s="43"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="44">
         <v>3</v>
       </c>
-      <c r="F29" s="35" t="s">
+      <c r="F29" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="G29" s="35" t="s">
+      <c r="G29" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="35" t="s">
+      <c r="H29" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="I29" s="35" t="s">
+      <c r="I29" s="38" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A30" s="31"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
+      <c r="A30" s="43"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="39"/>
+      <c r="I30" s="39"/>
     </row>
     <row r="31" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A31" s="31"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
+      <c r="A31" s="43"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43"/>
       <c r="E31" s="6">
         <v>4</v>
       </c>
@@ -1948,10 +1948,10 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A32" s="32"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="6">
         <v>5</v>
       </c>
@@ -1980,16 +1980,16 @@
       <c r="I33" s="7"/>
     </row>
     <row r="34" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="B34" s="35" t="s">
+      <c r="B34" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C34" s="35" t="s">
+      <c r="C34" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="D34" s="35" t="s">
+      <c r="D34" s="38" t="s">
         <v>95</v>
       </c>
       <c r="E34" s="3">
@@ -2009,10 +2009,10 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A35" s="31"/>
-      <c r="B35" s="31"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
+      <c r="A35" s="43"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
       <c r="E35" s="3">
         <v>2</v>
       </c>
@@ -2030,42 +2030,42 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A36" s="31"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="33">
+      <c r="A36" s="43"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="44">
         <v>3</v>
       </c>
-      <c r="F36" s="35" t="s">
+      <c r="F36" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="G36" s="35" t="s">
+      <c r="G36" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="H36" s="35" t="s">
+      <c r="H36" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="I36" s="35" t="s">
+      <c r="I36" s="38" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A37" s="31"/>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
+      <c r="A37" s="43"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
     </row>
     <row r="38" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A38" s="32"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
+      <c r="A38" s="39"/>
+      <c r="B38" s="39"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
       <c r="E38" s="8"/>
       <c r="F38" s="6"/>
       <c r="G38" s="4"/>
@@ -2084,16 +2084,16 @@
       <c r="I39" s="7"/>
     </row>
     <row r="40" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A40" s="35" t="s">
+      <c r="A40" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="B40" s="35" t="s">
+      <c r="B40" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="35" t="s">
+      <c r="C40" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="D40" s="35" t="s">
+      <c r="D40" s="38" t="s">
         <v>109</v>
       </c>
       <c r="E40" s="3">
@@ -2113,10 +2113,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A41" s="31"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
+      <c r="A41" s="43"/>
+      <c r="B41" s="43"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
       <c r="E41" s="3">
         <v>2</v>
       </c>
@@ -2134,32 +2134,32 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A42" s="31"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="35"/>
+      <c r="A42" s="43"/>
+      <c r="B42" s="43"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="43"/>
+      <c r="E42" s="44"/>
+      <c r="F42" s="45"/>
+      <c r="G42" s="47"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
     </row>
     <row r="43" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A43" s="31"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
+      <c r="A43" s="43"/>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="39"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="39"/>
+      <c r="I43" s="39"/>
     </row>
     <row r="44" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
+      <c r="A44" s="39"/>
+      <c r="B44" s="39"/>
+      <c r="C44" s="39"/>
+      <c r="D44" s="39"/>
       <c r="E44" s="6"/>
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
@@ -2178,16 +2178,16 @@
       <c r="I45" s="7"/>
     </row>
     <row r="46" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A46" s="35" t="s">
+      <c r="A46" s="38" t="s">
         <v>116</v>
       </c>
-      <c r="B46" s="35" t="s">
+      <c r="B46" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C46" s="35" t="s">
+      <c r="C46" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="35" t="s">
+      <c r="D46" s="38" t="s">
         <v>118</v>
       </c>
       <c r="E46" s="3">
@@ -2207,10 +2207,10 @@
       </c>
     </row>
     <row r="47" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A47" s="31"/>
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="31"/>
+      <c r="A47" s="43"/>
+      <c r="B47" s="43"/>
+      <c r="C47" s="43"/>
+      <c r="D47" s="43"/>
       <c r="E47" s="3">
         <v>2</v>
       </c>
@@ -2228,42 +2228,42 @@
       </c>
     </row>
     <row r="48" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A48" s="31"/>
-      <c r="B48" s="31"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="31"/>
-      <c r="E48" s="33">
+      <c r="A48" s="43"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="44">
         <v>3</v>
       </c>
-      <c r="F48" s="35" t="s">
+      <c r="F48" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="G48" s="35" t="s">
+      <c r="G48" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="H48" s="35" t="s">
+      <c r="H48" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="I48" s="35" t="s">
+      <c r="I48" s="38" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A49" s="31"/>
-      <c r="B49" s="31"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="31"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="32"/>
+      <c r="A49" s="43"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43"/>
+      <c r="E49" s="39"/>
+      <c r="F49" s="39"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="39"/>
+      <c r="I49" s="39"/>
     </row>
     <row r="50" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A50" s="32"/>
-      <c r="B50" s="32"/>
-      <c r="C50" s="32"/>
-      <c r="D50" s="32"/>
+      <c r="A50" s="39"/>
+      <c r="B50" s="39"/>
+      <c r="C50" s="39"/>
+      <c r="D50" s="39"/>
       <c r="E50" s="6">
         <v>4</v>
       </c>
@@ -2292,16 +2292,16 @@
       <c r="I51" s="7"/>
     </row>
     <row r="52" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="B52" s="35" t="s">
+      <c r="B52" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C52" s="35" t="s">
+      <c r="C52" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="D52" s="35" t="s">
+      <c r="D52" s="38" t="s">
         <v>134</v>
       </c>
       <c r="E52" s="3">
@@ -2321,10 +2321,10 @@
       </c>
     </row>
     <row r="53" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A53" s="31"/>
-      <c r="B53" s="31"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="31"/>
+      <c r="A53" s="43"/>
+      <c r="B53" s="43"/>
+      <c r="C53" s="43"/>
+      <c r="D53" s="43"/>
       <c r="E53" s="3">
         <v>2</v>
       </c>
@@ -2342,42 +2342,42 @@
       </c>
     </row>
     <row r="54" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A54" s="31"/>
-      <c r="B54" s="31"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="31"/>
-      <c r="E54" s="33">
+      <c r="A54" s="43"/>
+      <c r="B54" s="43"/>
+      <c r="C54" s="43"/>
+      <c r="D54" s="43"/>
+      <c r="E54" s="44">
         <v>3</v>
       </c>
-      <c r="F54" s="35" t="s">
+      <c r="F54" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="G54" s="35" t="s">
+      <c r="G54" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="H54" s="35" t="s">
+      <c r="H54" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="I54" s="35" t="s">
+      <c r="I54" s="38" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A55" s="31"/>
-      <c r="B55" s="31"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="31"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="32"/>
-      <c r="G55" s="32"/>
-      <c r="H55" s="32"/>
-      <c r="I55" s="32"/>
+      <c r="A55" s="43"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="43"/>
+      <c r="D55" s="43"/>
+      <c r="E55" s="39"/>
+      <c r="F55" s="39"/>
+      <c r="G55" s="39"/>
+      <c r="H55" s="39"/>
+      <c r="I55" s="39"/>
     </row>
     <row r="56" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A56" s="32"/>
-      <c r="B56" s="32"/>
-      <c r="C56" s="32"/>
-      <c r="D56" s="32"/>
+      <c r="A56" s="39"/>
+      <c r="B56" s="39"/>
+      <c r="C56" s="39"/>
+      <c r="D56" s="39"/>
       <c r="E56" s="6">
         <v>4</v>
       </c>
@@ -2406,16 +2406,16 @@
       <c r="I57" s="7"/>
     </row>
     <row r="58" spans="1:9" ht="43.2">
-      <c r="A58" s="35" t="s">
+      <c r="A58" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="B58" s="30" t="s">
+      <c r="B58" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C58" s="35" t="s">
+      <c r="C58" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="D58" s="35" t="s">
+      <c r="D58" s="38" t="s">
         <v>149</v>
       </c>
       <c r="E58" s="3">
@@ -2435,10 +2435,10 @@
       </c>
     </row>
     <row r="59" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A59" s="31"/>
-      <c r="B59" s="31"/>
-      <c r="C59" s="31"/>
-      <c r="D59" s="31"/>
+      <c r="A59" s="43"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="43"/>
       <c r="E59" s="3">
         <v>2</v>
       </c>
@@ -2456,11 +2456,11 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A60" s="31"/>
-      <c r="B60" s="31"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="31"/>
-      <c r="E60" s="33">
+      <c r="A60" s="43"/>
+      <c r="B60" s="43"/>
+      <c r="C60" s="43"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="44">
         <v>3</v>
       </c>
       <c r="F60" s="25" t="s">
@@ -2477,21 +2477,21 @@
       </c>
     </row>
     <row r="61" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A61" s="31"/>
-      <c r="B61" s="31"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="31"/>
-      <c r="E61" s="34"/>
+      <c r="A61" s="43"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="43"/>
+      <c r="D61" s="43"/>
+      <c r="E61" s="49"/>
       <c r="F61" s="27"/>
       <c r="G61" s="27"/>
       <c r="H61" s="27"/>
       <c r="I61" s="27"/>
     </row>
     <row r="62" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A62" s="31"/>
-      <c r="B62" s="31"/>
-      <c r="C62" s="31"/>
-      <c r="D62" s="31"/>
+      <c r="A62" s="43"/>
+      <c r="B62" s="43"/>
+      <c r="C62" s="43"/>
+      <c r="D62" s="43"/>
       <c r="E62" s="24"/>
       <c r="F62" s="28"/>
       <c r="G62" s="28"/>
@@ -2499,10 +2499,10 @@
       <c r="I62" s="28"/>
     </row>
     <row r="63" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A63" s="32"/>
-      <c r="B63" s="32"/>
-      <c r="C63" s="32"/>
-      <c r="D63" s="32"/>
+      <c r="A63" s="39"/>
+      <c r="B63" s="39"/>
+      <c r="C63" s="39"/>
+      <c r="D63" s="39"/>
       <c r="E63" s="24"/>
       <c r="F63" s="28"/>
       <c r="G63" s="28"/>
@@ -2521,16 +2521,16 @@
       <c r="I64" s="26"/>
     </row>
     <row r="65" spans="1:9" ht="43.2">
-      <c r="A65" s="30" t="s">
+      <c r="A65" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="B65" s="30" t="s">
+      <c r="B65" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C65" s="30" t="s">
+      <c r="C65" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="D65" s="30" t="s">
+      <c r="D65" s="48" t="s">
         <v>175</v>
       </c>
       <c r="E65" s="12">
@@ -2550,10 +2550,10 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="28.8">
-      <c r="A66" s="31"/>
-      <c r="B66" s="31"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="31"/>
+      <c r="A66" s="43"/>
+      <c r="B66" s="43"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
       <c r="E66" s="12">
         <v>2</v>
       </c>
@@ -2566,47 +2566,47 @@
       <c r="H66" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="I66" s="48" t="s">
+      <c r="I66" s="30" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A67" s="31"/>
-      <c r="B67" s="31"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="33">
+      <c r="A67" s="43"/>
+      <c r="B67" s="43"/>
+      <c r="C67" s="43"/>
+      <c r="D67" s="43"/>
+      <c r="E67" s="44">
         <v>3</v>
       </c>
-      <c r="F67" s="44" t="s">
+      <c r="F67" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="G67" s="44" t="s">
+      <c r="G67" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="H67" s="44" t="s">
+      <c r="H67" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="I67" s="44" t="s">
+      <c r="I67" s="32" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A68" s="31"/>
-      <c r="B68" s="31"/>
-      <c r="C68" s="31"/>
-      <c r="D68" s="31"/>
-      <c r="E68" s="32"/>
-      <c r="F68" s="45"/>
-      <c r="G68" s="45"/>
-      <c r="H68" s="45"/>
-      <c r="I68" s="45"/>
+      <c r="A68" s="43"/>
+      <c r="B68" s="43"/>
+      <c r="C68" s="43"/>
+      <c r="D68" s="43"/>
+      <c r="E68" s="39"/>
+      <c r="F68" s="33"/>
+      <c r="G68" s="33"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="33"/>
     </row>
     <row r="69" spans="1:9" ht="14.4">
-      <c r="A69" s="32"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="32"/>
-      <c r="D69" s="32"/>
+      <c r="A69" s="39"/>
+      <c r="B69" s="39"/>
+      <c r="C69" s="39"/>
+      <c r="D69" s="39"/>
       <c r="E69" s="8"/>
       <c r="F69" s="6"/>
       <c r="G69" s="4"/>
@@ -2625,16 +2625,16 @@
       <c r="I70" s="13"/>
     </row>
     <row r="71" spans="1:9" ht="34.200000000000003" customHeight="1">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="48" t="s">
         <v>173</v>
       </c>
-      <c r="B71" s="30" t="s">
+      <c r="B71" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C71" s="30" t="s">
+      <c r="C71" s="48" t="s">
         <v>184</v>
       </c>
-      <c r="D71" s="30" t="s">
+      <c r="D71" s="48" t="s">
         <v>185</v>
       </c>
       <c r="E71" s="12">
@@ -2654,14 +2654,14 @@
       </c>
     </row>
     <row r="72" spans="1:9" ht="28.8">
-      <c r="A72" s="31"/>
-      <c r="B72" s="31"/>
-      <c r="C72" s="31"/>
-      <c r="D72" s="31"/>
+      <c r="A72" s="43"/>
+      <c r="B72" s="43"/>
+      <c r="C72" s="43"/>
+      <c r="D72" s="43"/>
       <c r="E72" s="12">
         <v>2</v>
       </c>
-      <c r="F72" s="49" t="s">
+      <c r="F72" s="31" t="s">
         <v>190</v>
       </c>
       <c r="G72" s="15" t="s">
@@ -2675,42 +2675,42 @@
       </c>
     </row>
     <row r="73" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A73" s="31"/>
-      <c r="B73" s="31"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="31"/>
-      <c r="E73" s="46">
+      <c r="A73" s="43"/>
+      <c r="B73" s="43"/>
+      <c r="C73" s="43"/>
+      <c r="D73" s="43"/>
+      <c r="E73" s="34">
         <v>3</v>
       </c>
-      <c r="F73" s="50" t="s">
+      <c r="F73" s="36" t="s">
         <v>215</v>
       </c>
-      <c r="G73" s="51" t="s">
+      <c r="G73" s="37" t="s">
         <v>216</v>
       </c>
-      <c r="H73" s="51" t="s">
+      <c r="H73" s="37" t="s">
         <v>217</v>
       </c>
-      <c r="I73" s="51" t="s">
+      <c r="I73" s="37" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="39.6" customHeight="1">
-      <c r="A74" s="31"/>
-      <c r="B74" s="31"/>
-      <c r="C74" s="31"/>
-      <c r="D74" s="31"/>
-      <c r="E74" s="47"/>
-      <c r="F74" s="50"/>
-      <c r="G74" s="51"/>
-      <c r="H74" s="51"/>
-      <c r="I74" s="51"/>
+      <c r="A74" s="43"/>
+      <c r="B74" s="43"/>
+      <c r="C74" s="43"/>
+      <c r="D74" s="43"/>
+      <c r="E74" s="35"/>
+      <c r="F74" s="36"/>
+      <c r="G74" s="37"/>
+      <c r="H74" s="37"/>
+      <c r="I74" s="37"/>
     </row>
     <row r="75" spans="1:9" ht="21" customHeight="1">
-      <c r="A75" s="32"/>
-      <c r="B75" s="32"/>
-      <c r="C75" s="32"/>
-      <c r="D75" s="32"/>
+      <c r="A75" s="39"/>
+      <c r="B75" s="39"/>
+      <c r="C75" s="39"/>
+      <c r="D75" s="39"/>
       <c r="E75" s="19"/>
       <c r="F75" s="22"/>
       <c r="G75" s="21"/>
@@ -2729,16 +2729,16 @@
       <c r="I76" s="20"/>
     </row>
     <row r="77" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A77" s="30" t="s">
+      <c r="A77" s="48" t="s">
         <v>194</v>
       </c>
-      <c r="B77" s="35" t="s">
+      <c r="B77" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="C77" s="35" t="s">
+      <c r="C77" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="D77" s="35" t="s">
+      <c r="D77" s="38" t="s">
         <v>161</v>
       </c>
       <c r="E77" s="3">
@@ -2758,10 +2758,10 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A78" s="31"/>
-      <c r="B78" s="31"/>
-      <c r="C78" s="31"/>
-      <c r="D78" s="31"/>
+      <c r="A78" s="43"/>
+      <c r="B78" s="43"/>
+      <c r="C78" s="43"/>
+      <c r="D78" s="43"/>
       <c r="E78" s="3">
         <v>2</v>
       </c>
@@ -2779,42 +2779,42 @@
       </c>
     </row>
     <row r="79" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A79" s="31"/>
-      <c r="B79" s="31"/>
-      <c r="C79" s="31"/>
-      <c r="D79" s="31"/>
-      <c r="E79" s="33">
+      <c r="A79" s="43"/>
+      <c r="B79" s="43"/>
+      <c r="C79" s="43"/>
+      <c r="D79" s="43"/>
+      <c r="E79" s="44">
         <v>3</v>
       </c>
-      <c r="F79" s="35" t="s">
+      <c r="F79" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="G79" s="35" t="s">
+      <c r="G79" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="H79" s="35" t="s">
+      <c r="H79" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="I79" s="35" t="s">
+      <c r="I79" s="38" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A80" s="31"/>
-      <c r="B80" s="31"/>
-      <c r="C80" s="31"/>
-      <c r="D80" s="31"/>
-      <c r="E80" s="32"/>
-      <c r="F80" s="32"/>
-      <c r="G80" s="32"/>
-      <c r="H80" s="32"/>
-      <c r="I80" s="32"/>
+      <c r="A80" s="43"/>
+      <c r="B80" s="43"/>
+      <c r="C80" s="43"/>
+      <c r="D80" s="43"/>
+      <c r="E80" s="39"/>
+      <c r="F80" s="39"/>
+      <c r="G80" s="39"/>
+      <c r="H80" s="39"/>
+      <c r="I80" s="39"/>
     </row>
     <row r="81" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A81" s="32"/>
-      <c r="B81" s="32"/>
-      <c r="C81" s="32"/>
-      <c r="D81" s="32"/>
+      <c r="A81" s="39"/>
+      <c r="B81" s="39"/>
+      <c r="C81" s="39"/>
+      <c r="D81" s="39"/>
       <c r="E81" s="8"/>
       <c r="F81" s="6"/>
       <c r="G81" s="4"/>
@@ -3752,62 +3752,51 @@
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="115">
-    <mergeCell ref="I67:I68"/>
-    <mergeCell ref="H67:H68"/>
-    <mergeCell ref="G67:G68"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="G73:G74"/>
-    <mergeCell ref="H73:H74"/>
-    <mergeCell ref="I73:I74"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="D3:D7"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="C9:C13"/>
-    <mergeCell ref="D9:D13"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="A15:A19"/>
-    <mergeCell ref="B15:B19"/>
-    <mergeCell ref="C15:C19"/>
-    <mergeCell ref="D15:D19"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H42:H43"/>
-    <mergeCell ref="I42:I43"/>
-    <mergeCell ref="A40:A44"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="C40:C44"/>
-    <mergeCell ref="D40:D44"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="H48:H49"/>
-    <mergeCell ref="I48:I49"/>
-    <mergeCell ref="A46:A50"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="C46:C50"/>
-    <mergeCell ref="D46:D50"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="A71:A75"/>
+    <mergeCell ref="B71:B75"/>
+    <mergeCell ref="C71:C75"/>
+    <mergeCell ref="D71:D75"/>
+    <mergeCell ref="A65:A69"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="C65:C69"/>
+    <mergeCell ref="D65:D69"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="H79:H80"/>
+    <mergeCell ref="I79:I80"/>
+    <mergeCell ref="A77:A81"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="C77:C81"/>
+    <mergeCell ref="D77:D81"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="G79:G80"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="A34:A38"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="C34:C38"/>
+    <mergeCell ref="D34:D38"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="G36:G37"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="C27:C32"/>
+    <mergeCell ref="D27:D32"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="D21:D25"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
     <mergeCell ref="A58:A63"/>
     <mergeCell ref="B58:B63"/>
     <mergeCell ref="C58:C63"/>
@@ -3822,51 +3811,62 @@
     <mergeCell ref="E54:E55"/>
     <mergeCell ref="F54:F55"/>
     <mergeCell ref="G54:G55"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="B21:B25"/>
-    <mergeCell ref="C21:C25"/>
-    <mergeCell ref="D21:D25"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="C27:C32"/>
-    <mergeCell ref="D27:D32"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="A34:A38"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="G36:G37"/>
-    <mergeCell ref="H79:H80"/>
-    <mergeCell ref="I79:I80"/>
-    <mergeCell ref="A77:A81"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="C77:C81"/>
-    <mergeCell ref="D77:D81"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="G79:G80"/>
-    <mergeCell ref="A71:A75"/>
-    <mergeCell ref="B71:B75"/>
-    <mergeCell ref="C71:C75"/>
-    <mergeCell ref="D71:D75"/>
-    <mergeCell ref="A65:A69"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="C65:C69"/>
-    <mergeCell ref="D65:D69"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="H48:H49"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="A46:A50"/>
+    <mergeCell ref="B46:B50"/>
+    <mergeCell ref="C46:C50"/>
+    <mergeCell ref="D46:D50"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="H42:H43"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="C40:C44"/>
+    <mergeCell ref="D40:D44"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="C15:C19"/>
+    <mergeCell ref="D15:D19"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="C9:C13"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="D3:D7"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="I67:I68"/>
+    <mergeCell ref="H67:H68"/>
+    <mergeCell ref="G67:G68"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="G73:G74"/>
+    <mergeCell ref="H73:H74"/>
+    <mergeCell ref="I73:I74"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>